<commit_message>
update: input arguments to execute the dispatcher or/and performer process to demand. additionaly, added integration with Open AI to solve some questions about location and keywords into the offer description.
</commit_message>
<xml_diff>
--- a/Linkedin_Process/Data/Config.xlsx
+++ b/Linkedin_Process/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Documents\UiPath\RPA_Projects\Linkedin_Process\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57BE0E0B-FCE2-489A-9817-2E484B7D27C3}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3246603-5BC1-442D-82E0-968D17FF3FA2}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="732" yWindow="732" windowWidth="13812" windowHeight="10464" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1152" yWindow="1152" windowWidth="23220" windowHeight="8832" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="54">
   <si>
     <t>Name</t>
   </si>
@@ -172,6 +172,21 @@
   </si>
   <si>
     <t>Linkedin_StorageBucketName</t>
+  </si>
+  <si>
+    <t>Linkedin_RoleNames</t>
+  </si>
+  <si>
+    <t>ListRoleName</t>
+  </si>
+  <si>
+    <t>UserSettingsPathFile</t>
+  </si>
+  <si>
+    <t>Data\UserSettings.xlsx</t>
+  </si>
+  <si>
+    <t>File with keywords that we expect to find into jobOfferDetail</t>
   </si>
 </sst>
 </file>
@@ -624,7 +639,17 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="6" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" t="s">
+        <v>53</v>
+      </c>
+    </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
@@ -2837,7 +2862,14 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="3" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A3" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" t="s">
+        <v>49</v>
+      </c>
+    </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="5" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
@@ -3838,5 +3870,6 @@
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>